<commit_message>
feat(F-NAR-019): ATOM-DIF.BES.001-07 Victorina observe d'abord les cartes
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.BES.001-07.xlsx
+++ b/stories/arbres/ATOM-DIF.BES.001-07.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>La poire du magasin</t>
+          <t>Victorina observe d'abord les cartes</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>véranda, draps au soleil</t>
+          <t>classe, rayon de soleil, poussière, chaises de bois, table basse, cartes, horloge, foulard au crochet</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Victorina, Chouchou, papa, maman</t>
+          <t>Victorina, papa, maman</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Victorina veut la poire de bois du magasin en carton. Elle reste près de l'escalier. Chouchou répète : un fruit, on dit le nom. Elle observe d'abord, puis montre la poire. La clochette ferme le magasin.</t>
+          <t>Un rayon coupe la classe. La poussière flotte. Dans le rayon, un éclat de poussière brille. Victorina veut montrer la pomme maintenant. Sa voix part trop fort : les cartes glissent. Elle refuse de foncer, observe, dit le mot plus bas. On le dit comme elle. Merci vécu. Un éclat de poussière reste pâle.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Des draps blancs sèchent sur la véranda. Le soleil passe à travers le linge. Ça fait des taches chaudes au sol. Une pince à linge claque, tout doux. Ça sent le savon, tout près. Un carton ouvert sert de magasin. Dessus, des fruits de bois. Une pomme. Une banane. Une poire claire. Une clochette attend dans une chaussette. Tu as senti le drap, Victorina ? Oui, papa. Il est encore un peu humide. On parle tout doux, d'accord ? D'accord. En ce moment, Chouchou pose la pomme. Le bois est lisse et tiède. Le magasin est ouvert. Un fruit. On dit le nom. Victorina reste près de l'escalier. Le bois de l'escalier est frais. Elle a besoin de calme. La poire est pour moi. Ses mains restent sur la rampe. Victorina. Tu viens ? Victorina ne vient pas encore. On peut répéter la règle. On peut observer d'abord. D'accord. Chouchou va près de l'escalier. Il parle tout bas. La clochette bouge dans la chaussette. Tu as entendu la clochette ? Un tout petit peu. Elle est dans la chaussette. Elle sonne moins fort. Victorina regarde la poire. La poire a une petite feuille peinte. Elle est claire. Oui. Elle attend.</t>
+          <t>Un rayon coupe la classe, pâle et droit. La poussière flotte, lente. Dans le rayon, un éclat de poussière brille. Il brille, papa. Tu le vois, dans l'air ? Les chaises de bois font un petit bruit. Elles craquent. C'est le bois des chaises. Le foulard de maman pend au crochet. Il est bleu. Il pend au crochet. Tu restes près de nous, Victorina ? Oui, papa. L'horloge fait tic, puis tac. Je l'entends. Elle compte, sans se presser. Le mur est frais, près du crochet. Il est frais, papa. Oui, le mur de la classe. Une table basse attend au milieu. Des cartes y sont posées, faces ouvertes. La pomme rouge, maman ! Tu la vois, sur la table ? Une carte montre une pomme, bien ronde. Elle est rouge. À côté, un canard garde le bec fermé. Un chat aux oreilles hautes attend aussi. Le chat me regarde. Ils sont tous sur la table. Victorina touche l'éclat de poussière. L'air est tiède, un peu piquant. Ça chatouille le nez. Je la montre, maintenant ! Tu restes près de la table ? Oui, maman. La classe est trop grande, pour crier. Je parle fort, alors. En ce moment, Victorina se penche sur la table. Pomme, tu vas dans le rayon ! Sa voix part trop fort, trop vite. Les chaises de bois reculent d'un coup. Les cartes glissent sur la table. Oh. La pomme disparaît sous le canard. L'éclat n'est plus là. Le sourire de Victorina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je la prends ! La pomme est sous les autres. Tu la vois, Victorina ? Les épaules de Victorina tombent un peu. Ça serre, dans son ventre. Papa se baisse à sa hauteur.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Des draps blancs sèchent sur la véranda. Le soleil passe à travers le linge. Ça fait des taches chaudes au sol. Une pince à linge claque, tout doux. Ça sent le savon, tout près. Un carton ouvert sert de magasin. Dessus, des fruits de bois. Une pomme. Une banane. Une poire claire. Une clochette attend dans une chaussette. Tu as senti le drap, Victorina ? Oui, papa. Il est encore un peu humide. On parle tout doux, d'accord ? D'accord. En ce moment, Chouchou pose la pomme. Le bois est lisse et tiède. Le magasin est ouvert. Un fruit. On dit le nom. Victorina reste près de l'escalier. Le bois de l'escalier est frais. Elle a besoin de calme. La poire est pour moi. Ses mains restent sur la rampe. Victorina. Tu viens ? Victorina ne vient pas encore. On peut répéter la règle. On peut observer d'abord. D'accord. Chouchou va près de l'escalier. Il parle tout bas. La clochette bouge dans la chaussette. Tu as entendu la clochette ? Un tout petit peu. Elle est dans la chaussette. Elle sonne moins fort. Victorina regarde la poire. La poire a une petite feuille peinte. Elle est claire. Oui. Elle attend.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un rayon coupe la classe, pâle et droit. La poussière flotte, lente. Dans le rayon, un &lt;emphasis level="moderate"&gt;éclat de poussière&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, dans l'air ? Les chaises de bois font un petit bruit. Elles craquent. C'est le bois des chaises. Le foulard de maman pend au crochet. Il est bleu. Il pend au crochet. Tu restes près de nous, Victorina ? Oui, papa. L'horloge fait tic, puis tac. Je l'entends. Elle compte, sans se presser. Le mur est frais, près du crochet. Il est frais, papa. Oui, le mur de la classe. Une table basse attend au milieu. Des cartes y sont posées, faces ouvertes. La pomme rouge, maman ! Tu la vois, sur la table ? Une carte montre une pomme, bien ronde. Elle est rouge. À côté, un canard garde le bec fermé. Un chat aux oreilles hautes attend aussi. Le chat me regarde. Ils sont tous sur la table. Victorina touche l'éclat de poussière. L'air est tiède, un peu piquant. Ça chatouille le nez. Je la montre, maintenant ! Tu restes près de la table ? Oui, maman. La classe est trop grande, pour crier. Je parle fort, alors. En ce moment, Victorina se penche sur la table. Pomme, tu vas dans le rayon ! Sa voix part trop fort, trop vite. Les chaises de bois reculent d'un coup. Les cartes glissent sur la table. Oh. La pomme disparaît sous le canard. L'éclat n'est plus là. Le sourire de Victorina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je la prends ! La pomme est sous les autres. Tu la vois, Victorina ? Les épaules de Victorina tombent un peu. Ça serre, dans son ventre. Papa se baisse à sa hauteur.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Anaïs est en classe. Corentin explique un jeu de cartes. Anaïs reste près du mur. Elle a besoin de calme. Corentin va &lt;emphasis&gt;répéter&lt;/emphasis&gt; la règle. Il dit : on pioche. On montre. Anaïs écoute. Elle va observer d'abord. Elle regarde. Elle ne joue pas encore. La maîtresse dit : observer d'abord, c'est possible. Plus tard, Anaïs pioche une carte. Le soir, maman dit : tu as su répéter. Anaïs a pu observer d'abord. [pause]</t>
+          <t>Un rayon coupe la classe, pâle et droit. La poussière flotte, lente. Dans le rayon, un &lt;emphasis&gt;éclat de poussière&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, dans l'air ? Les chaises de bois font un petit bruit. Elles craquent. C'est le bois des chaises. Le foulard de maman pend au crochet. Il est bleu. Il pend au crochet. Tu restes près de nous, Victorina ? Oui, papa. L'horloge fait tic, puis tac. Je l'entends. Elle compte, sans se presser. Le mur est frais, près du crochet. Il est frais, papa. Oui, le mur de la classe. Une table basse attend au milieu. Des cartes y sont posées, faces ouvertes. La pomme rouge, maman ! Tu la vois, sur la table ? Une carte montre une pomme, bien ronde. Elle est rouge. À côté, un canard garde le bec fermé. Un chat aux oreilles hautes attend aussi. Le chat me regarde. Ils sont tous sur la table. Victorina touche l'éclat de poussière. L'air est tiède, un peu piquant. Ça chatouille le nez. Je la montre, maintenant ! Tu restes près de la table ? Oui, maman. La classe est trop grande, pour crier. Je parle fort, alors. En ce moment, Victorina se penche sur la table. Pomme, tu vas dans le rayon ! Sa voix part trop fort, trop vite. Les chaises de bois reculent d'un coup. Les cartes glissent sur la table. Oh. La pomme disparaît sous le canard. L'éclat n'est plus là. Le sourire de Victorina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je la prends ! La pomme est sous les autres. Tu la vois, Victorina ? Les épaules de Victorina tombent un peu. Ça serre, dans son ventre. Papa se baisse à sa hauteur. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>répéter</t>
+          <t>éclat de poussière</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,58 +1326,71 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience_curieuse puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_montrer_la_pomme_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Des draps blancs sèchent sur la véranda.
-narrateur|Le soleil passe à travers le linge.
-narrateur|Ça fait des taches chaudes au sol.
-narrateur|Une pince à linge claque, tout doux.
-narrateur|Ça sent le savon, tout près.
-narrateur|Un carton ouvert sert de magasin.
-narrateur|Dessus, des fruits de bois.
-narrateur|Une pomme.
-narrateur|Une banane.
-narrateur|Une poire claire.
-narrateur|Une clochette attend dans une chaussette.
-papa|Tu as senti le drap, Victorina ?
+          <t>narrateur|Un rayon coupe la classe, pâle et droit.
+narrateur|La poussière flotte, lente.
+narrateur|Dans le rayon, un éclat de poussière brille.
+enfant-f|Il brille, papa.
+papa|Tu le vois, dans l'air ?
+narrateur|Les chaises de bois font un petit bruit.
+enfant-f|Elles craquent.
+maman|C'est le bois des chaises.
+narrateur|Le foulard de maman pend au crochet.
+enfant-f|Il est bleu.
+maman|Il pend au crochet.
+papa|Tu restes près de nous, Victorina ?
 enfant-f|Oui, papa.
-enfant-f|Il est encore un peu humide.
-maman|On parle tout doux, d'accord ?
-enfant-f|D'accord.
-narrateur|En ce moment, Chouchou pose la pomme.
-narrateur|Le bois est lisse et tiède.
-copain|Le magasin est ouvert.
-copain|Un fruit.
-copain|On dit le nom.
-narrateur|Victorina reste près de l'escalier.
-narrateur|Le bois de l'escalier est frais.
-narrateur|Elle a besoin de calme.
-enfant-f|La poire est pour moi.
-narrateur|Ses mains restent sur la rampe.
-copain|Victorina.
-copain|Tu viens ?
-narrateur|Victorina ne vient pas encore.
-papa|On peut répéter la règle.
-maman|On peut observer d'abord.
-copain|D'accord.
-narrateur|Chouchou va près de l'escalier.
-narrateur|Il parle tout bas.
-narrateur|La clochette bouge dans la chaussette.
-papa|Tu as entendu la clochette ?
-enfant-f|Un tout petit peu.
-maman|Elle est dans la chaussette.
-maman|Elle sonne moins fort.
-narrateur|Victorina regarde la poire.
-narrateur|La poire a une petite feuille peinte.
-enfant-f|Elle est claire.
-papa|Oui.
-papa|Elle attend.</t>
+narrateur|L'horloge fait tic, puis tac.
+enfant-f|Je l'entends.
+papa|Elle compte, sans se presser.
+narrateur|Le mur est frais, près du crochet.
+enfant-f|Il est frais, papa.
+papa|Oui, le mur de la classe.
+narrateur|Une table basse attend au milieu.
+narrateur|Des cartes y sont posées, faces ouvertes.
+enfant-f|La pomme rouge, maman !
+maman|Tu la vois, sur la table ?
+narrateur|Une carte montre une pomme, bien ronde.
+enfant-f|Elle est rouge.
+narrateur|À côté, un canard garde le bec fermé.
+narrateur|Un chat aux oreilles hautes attend aussi.
+enfant-f|Le chat me regarde.
+papa|Ils sont tous sur la table.
+narrateur|Victorina touche l'éclat de poussière.
+narrateur|L'air est tiède, un peu piquant.
+enfant-f|Ça chatouille le nez.
+enfant-f|Je la montre, maintenant !
+maman|Tu restes près de la table ?
+enfant-f|Oui, maman.
+papa|La classe est trop grande, pour crier.
+enfant-f|Je parle fort, alors.
+narrateur|En ce moment, Victorina se penche sur la table.
+enfant-f|Pomme, tu vas dans le rayon !
+narrateur|Sa voix part trop fort, trop vite.
+narrateur|Les chaises de bois reculent d'un coup.
+narrateur|Les cartes glissent sur la table.
+enfant-f|Oh.
+narrateur|La pomme disparaît sous le canard.
+narrateur|L'éclat n'est plus là.
+narrateur|Le sourire de Victorina disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+enfant-f|Je la prends !
+maman|La pomme est sous les autres.
+papa|Tu la vois, Victorina ?
+narrateur|Les épaules de Victorina tombent un peu.
+narrateur|Ça serre, dans son ventre.
+narrateur|Papa se baisse à sa hauteur.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>draps,bois</t>
+          <t>chaises,rayon</t>
         </is>
       </c>
     </row>
@@ -1409,12 +1422,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Victorina a besoin de calme. Que peut-on faire ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Victorina a besoin de &lt;emphasis level="moderate"&gt;calme&lt;/emphasis&gt;. Que peut-on faire ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Anaïs a besoin de calme. Que peut-on faire ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Victorina a besoin de &lt;emphasis&gt;calme&lt;/emphasis&gt;. Que peut-on faire ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1439,7 +1452,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>On répète la règle. Victorina peut quoi d'abord ?</t>
+          <t>On peut répéter. Que peut-on faire ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1477,7 +1490,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1488,7 +1501,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1503,34 +1516,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1545,17 +1562,17 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=on_dit_le_mot_une_seconde_fois; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1588,17 +1605,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Chouchou répète, tout bas. Un fruit. On dit le nom. Victorina écoute. Elle va observer d'abord. Elle regarde la pomme. Pomme. Il la pose sur le carton. Ça fait un petit toc. Observer d'abord, c'est possible. Victorina avance un pied. Puis elle s'arrête. Tu vois la poire, Victorina ? Oui. La petite feuille. Chouchou montre la banane. Banane. Victorina suit des yeux. Elle ne prend pas encore. Tu as répété, Chouchou ? Oui. Victorina peut regarder. Un coin de drap claque un peu. Le soleil a bougé.</t>
+          <t>Victorina avance trop vite vers la table. Pomme, maintenant ! Sa voix se mélange au bruit des chaises. Oh. Les cartes restent en tas. Elle refuse de foncer. Victorina referme la main. Elle regarde la table, un instant. Tu veux venir près de la pomme ? Papa s'accroupit à la même hauteur. Victorina pose un genou près de la table. La table est lisse, un peu froide. Pomme. Elle dit le mot plus bas. Pomme. Papa dit le mot, comme elle. Pomme. Victorina dit le mot, une seconde fois. Merci, Victorina. Maman a entendu toute la phrase. Le ventre de Victorina se desserre. Les épaules se relèvent un peu. Tu as les mains au chaud ? Un peu, papa. L'horloge fait tic, puis tac. Elle va moins vite. Tu l'entends, Victorina ? Oui. Victorina écarte les cartes, sans les jeter. La pomme revient, sur le papier. Elle est là. Elle t'écoute. Victorina pose un doigt près de la pomme. Le papier est un peu froid. Tu la montres dans le rayon ? Oui, papa.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Chouchou répète, tout bas. Un fruit. On dit le nom. Victorina écoute. Elle va observer d'abord. Elle regarde la pomme. Pomme. Il la pose sur le carton. Ça fait un petit toc. Observer d'abord, c'est possible. Victorina avance un pied. Puis elle s'arrête. Tu vois la poire, Victorina ? Oui. La petite feuille. Chouchou montre la banane. Banane. Victorina suit des yeux. Elle ne prend pas encore. Tu as répété, Chouchou ? Oui. Victorina peut regarder. Un coin de drap claque un peu. Le soleil a bougé.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Victorina avance trop vite vers la table. &lt;emphasis level="moderate"&gt;Pomme&lt;/emphasis&gt;, maintenant ! Sa voix se mélange au bruit des chaises. Oh. Les cartes restent en tas. Elle refuse de foncer. Victorina referme la main. Elle regarde la table, un instant. Tu veux venir près de la pomme ? Papa s'accroupit à la même hauteur. Victorina pose un genou près de la table. La table est lisse, un peu froide. Pomme. Elle dit le mot plus bas. Pomme. Papa dit le mot, comme elle. Pomme. Victorina dit le mot, une seconde fois. Merci, Victorina. Maman a entendu toute la phrase. Le ventre de Victorina se desserre. Les épaules se relèvent un peu. Tu as les mains au chaud ? Un peu, papa. L'horloge fait tic, puis tac. Elle va moins vite. Tu l'entends, Victorina ? Oui. Victorina écarte les cartes, sans les jeter. La pomme revient, sur le papier. Elle est là. Elle t'écoute. Victorina pose un doigt près de la pomme. Le papier est un peu froid. Tu la montres dans le rayon ? Oui, papa.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Corentin a répété. Anaïs a observé d'abord. Puis elle a joué un peu. [pause]</t>
+          <t>Victorina avance trop vite vers la table. &lt;emphasis&gt;Pomme&lt;/emphasis&gt;, maintenant ! Sa voix se mélange au bruit des chaises. Oh. Les cartes restent en tas. Elle refuse de foncer. Victorina referme la main. Elle regarde la table, un instant. Tu veux venir près de la pomme ? Papa s'accroupit à la même hauteur. Victorina pose un genou près de la table. La table est lisse, un peu froide. Pomme. Elle dit le mot plus bas. Pomme. Papa dit le mot, comme elle. Pomme. Victorina dit le mot, une seconde fois. Merci, Victorina. Maman a entendu toute la phrase. Le ventre de Victorina se desserre. Les épaules se relèvent un peu. Tu as les mains au chaud ? Un peu, papa. L'horloge fait tic, puis tac. Elle va moins vite. Tu l'entends, Victorina ? Oui. Victorina écarte les cartes, sans les jeter. La pomme revient, sur le papier. Elle est là. Elle t'écoute. Victorina pose un doigt près de la pomme. Le papier est un peu froid. Tu la montres dans le rayon ? Oui, papa. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1656,7 +1673,7 @@
         <v>0.92</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.2</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1677,7 +1694,11 @@
       <c r="AG4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH4" s="2" t="inlineStr"/>
+      <c r="AH4" s="2" t="inlineStr">
+        <is>
+          <t>Pomme</t>
+        </is>
+      </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
@@ -1689,16 +1710,16 @@
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1723,40 +1744,52 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=confirmation; intention=relancer; emotion=soulagement_prudent; intensite=1; destinataire=enfant; sous_texte=la_voix_forte_echoue_le_mot_revient_plus_bas; tempo=naturel; sourire=léger; respiration=fluide</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Chouchou répète, tout bas.
-copain|Un fruit.
-copain|On dit le nom.
-narrateur|Victorina écoute.
-narrateur|Elle va observer d'abord.
-narrateur|Elle regarde la pomme.
-copain|Pomme.
-narrateur|Il la pose sur le carton.
-narrateur|Ça fait un petit toc.
-maman|Observer d'abord, c'est possible.
-narrateur|Victorina avance un pied.
-narrateur|Puis elle s'arrête.
-papa|Tu vois la poire, Victorina ?
+          <t>narrateur|Victorina avance trop vite vers la table.
+enfant-f|Pomme, maintenant !
+narrateur|Sa voix se mélange au bruit des chaises.
+enfant-f|Oh.
+narrateur|Les cartes restent en tas.
+narrateur|Elle refuse de foncer.
+narrateur|Victorina referme la main.
+narrateur|Elle regarde la table, un instant.
+papa|Tu veux venir près de la pomme ?
+narrateur|Papa s'accroupit à la même hauteur.
+narrateur|Victorina pose un genou près de la table.
+narrateur|La table est lisse, un peu froide.
+enfant-f|Pomme.
+narrateur|Elle dit le mot plus bas.
+papa|Pomme.
+narrateur|Papa dit le mot, comme elle.
+enfant-f|Pomme.
+narrateur|Victorina dit le mot, une seconde fois.
+maman|Merci, Victorina.
+narrateur|Maman a entendu toute la phrase.
+narrateur|Le ventre de Victorina se desserre.
+narrateur|Les épaules se relèvent un peu.
+papa|Tu as les mains au chaud ?
+enfant-f|Un peu, papa.
+narrateur|L'horloge fait tic, puis tac.
+enfant-f|Elle va moins vite.
+papa|Tu l'entends, Victorina ?
 enfant-f|Oui.
-enfant-f|La petite feuille.
-narrateur|Chouchou montre la banane.
-copain|Banane.
-narrateur|Victorina suit des yeux.
-narrateur|Elle ne prend pas encore.
-maman|Tu as répété, Chouchou ?
-copain|Oui.
-papa|Victorina peut regarder.
-narrateur|Un coin de drap claque un peu.
-narrateur|Le soleil a bougé.</t>
+narrateur|Victorina écarte les cartes, sans les jeter.
+narrateur|La pomme revient, sur le papier.
+enfant-f|Elle est là.
+maman|Elle t'écoute.
+narrateur|Victorina pose un doigt près de la pomme.
+narrateur|Le papier est un peu froid.
+papa|Tu la montres dans le rayon ?
+enfant-f|Oui, papa.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
         <is>
-          <t>bois</t>
+          <t>chaises,cartes</t>
         </is>
       </c>
     </row>
@@ -1783,17 +1816,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, Victorina tend la main. Elle prend la poire de bois. Elle la montre, tout doux. Poire. Oui. Elle pose la poire sur le carton. Tu as observé d'abord. Bravo, Chouchou. Tu as répété tout bas. Chouchou sort la clochette. Il la secoue une fois. Ça fait un son mou. Le magasin ferme ? Oui. La poire reste. Tu as fini ta poire ? Oui, papa. Les draps bougent encore. Ça sent toujours le savon.</t>
+          <t>Victorina tire la carte trop vite. Tu vas dans le rayon, d'un coup ! La carte glisse sous une chaise de bois. Oh. Victorina avance la main. Puis elle s'arrête net. Attends, je regarde. Papa attend, sans parler. Victorina observe la table, écoute la classe. Dans le rayon, un éclat de poussière luit. Là, près du foulard. Victorina tient la carte des deux mains. Le papier est lisse, un peu froid. Elle est froide, papa. Tu la portes jusqu'au rayon ? Oui, papa. On avance ? Oui, maman. Victorina pose la pomme dans le rayon pâle. Le papier touche l'air tiède. L'air tiède revient sur les joues. Victorina serre la carte contre elle. Elle reste froide. On marche. La carte penche, puis se cale. Je la tiens. On avance. Victorina passe le long des chaises. Le bois craque, un peu. Je la tiens bien. On marche près du crochet. Le foulard est là.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, Victorina tend la main. Elle prend la poire de bois. Elle la montre, tout doux. Poire. Oui. Elle pose la poire sur le carton. Tu as observé d'abord. Bravo, Chouchou. Tu as répété tout bas. Chouchou sort la clochette. Il la secoue une fois. Ça fait un son mou. Le magasin ferme ? Oui. La poire reste. Tu as fini ta poire ? Oui, papa. Les draps bougent encore. Ça sent toujours le savon.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Victorina tire la carte trop vite. Tu vas dans le rayon, d'un coup ! La carte glisse sous une chaise de bois. Oh. Victorina avance la main. Puis elle s'arrête net. Attends, je regarde. Papa attend, sans parler. Victorina observe la table, écoute la classe. Dans le rayon, un &lt;emphasis level="moderate"&gt;éclat de poussière&lt;/emphasis&gt; luit. Là, près du foulard. Victorina tient la carte des deux mains. Le papier est lisse, un peu froid. Elle est froide, papa. Tu la portes jusqu'au rayon ? Oui, papa. On avance ? Oui, maman. Victorina pose la pomme dans le rayon pâle. Le papier touche l'air tiède. L'air tiède revient sur les joues. Victorina serre la carte contre elle. Elle reste froide. On marche. La carte penche, puis se cale. Je la tiens. On avance. Victorina passe le long des chaises. Le bois craque, un peu. Je la tiens bien. On marche près du crochet. Le foulard est là.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Maman range le cartable. Anaïs donne la &lt;emphasis&gt;main&lt;/emphasis&gt;. [pause]</t>
+          <t>Victorina tire la carte trop vite. Tu vas dans le rayon, d'un coup ! La carte glisse sous une chaise de bois. Oh. Victorina avance la main. Puis elle s'arrête net. Attends, je regarde. Papa attend, sans parler. Victorina observe la table, écoute la classe. Dans le rayon, un &lt;emphasis&gt;éclat de poussière&lt;/emphasis&gt; luit. Là, près du foulard. Victorina tient la carte des deux mains. Le papier est lisse, un peu froid. Elle est froide, papa. Tu la portes jusqu'au rayon ? Oui, papa. On avance ? Oui, maman. Victorina pose la pomme dans le rayon pâle. Le papier touche l'air tiède. L'air tiède revient sur les joues. Victorina serre la carte contre elle. Elle reste froide. On marche. La carte penche, puis se cale. Je la tiens. On avance. Victorina passe le long des chaises. Le bois craque, un peu. Je la tiens bien. On marche près du crochet. Le foulard est là. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1840,7 +1873,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1848,10 +1881,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1874,30 +1907,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de poussière</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1906,10 +1939,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1920,33 +1953,50 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_sans_regarder_l_eclat; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Plus tard, Victorina tend la main.
-narrateur|Elle prend la poire de bois.
-narrateur|Elle la montre, tout doux.
-enfant-f|Poire.
-copain|Oui.
-narrateur|Elle pose la poire sur le carton.
-papa|Tu as observé d'abord.
-maman|Bravo, Chouchou.
-maman|Tu as répété tout bas.
-narrateur|Chouchou sort la clochette.
-narrateur|Il la secoue une fois.
-narrateur|Ça fait un son mou.
-enfant-f|Le magasin ferme ?
-copain|Oui.
-copain|La poire reste.
-papa|Tu as fini ta poire ?
+          <t>narrateur|Victorina tire la carte trop vite.
+enfant-f|Tu vas dans le rayon, d'un coup !
+narrateur|La carte glisse sous une chaise de bois.
+enfant-f|Oh.
+narrateur|Victorina avance la main.
+narrateur|Puis elle s'arrête net.
+enfant-f|Attends, je regarde.
+narrateur|Papa attend, sans parler.
+narrateur|Victorina observe la table, écoute la classe.
+narrateur|Dans le rayon, un éclat de poussière luit.
+enfant-f|Là, près du foulard.
+narrateur|Victorina tient la carte des deux mains.
+narrateur|Le papier est lisse, un peu froid.
+enfant-f|Elle est froide, papa.
+papa|Tu la portes jusqu'au rayon ?
 enfant-f|Oui, papa.
-narrateur|Les draps bougent encore.
-narrateur|Ça sent toujours le savon.</t>
+maman|On avance ?
+enfant-f|Oui, maman.
+narrateur|Victorina pose la pomme dans le rayon pâle.
+narrateur|Le papier touche l'air tiède.
+narrateur|L'air tiède revient sur les joues.
+narrateur|Victorina serre la carte contre elle.
+enfant-f|Elle reste froide.
+papa|On marche.
+narrateur|La carte penche, puis se cale.
+enfant-f|Je la tiens.
+maman|On avance.
+narrateur|Victorina passe le long des chaises.
+narrateur|Le bois craque, un peu.
+enfant-f|Je la tiens bien.
+papa|On marche près du crochet.
+enfant-f|Le foulard est là.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>clochette</t>
+          <t>chaises,rayon</t>
         </is>
       </c>
     </row>
@@ -1973,17 +2023,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>La poire claire brille sur le carton. J'ai regardé d'abord. J'ai répété. Puis la poire est arrivée. Oui. La clochette dort dans la chaussette.</t>
+          <t>Le rayon brillait, papa. Tu le vois, comme dans l'air ? Oui, un peu pâle. Victorina pose la carte contre le foulard. On la garde près de nous ? Oui, maman. La classe sentait le bois. Elle est derrière nous. Un rayon n'est plus aussi net. Victorina respire, plus large. On rentre ? Oui. Les joues de Victorina se réchauffent. La carte reste froide sous la main. On le voit, maman. Tu le vois dans l'air ? Oui, l'éclat. Un éclat de poussière reste pâle.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>La poire claire brille sur le carton. J'ai regardé d'abord. J'ai répété. Puis la poire est arrivée. Oui. La clochette dort dans la chaussette.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le rayon brillait, papa. Tu le vois, comme dans l'air ? Oui, un peu pâle. Victorina pose la carte contre le foulard. On la garde près de nous ? Oui, maman. La classe sentait le bois. Elle est derrière nous. Un rayon n'est plus aussi net. Victorina respire, plus large. On rentre ? Oui. Les joues de Victorina se réchauffent. La carte reste froide sous la main. On le voit, maman. Tu le vois dans l'air ? Oui, l'éclat. Un &lt;emphasis level="moderate"&gt;éclat de poussière&lt;/emphasis&gt; reste pâle.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le rayon brillait, papa. Tu le vois, comme dans l'air ? Oui, un peu pâle. Victorina pose la carte contre le foulard. On la garde près de nous ? Oui, maman. La classe sentait le bois. Elle est derrière nous. Un rayon n'est plus aussi net. Victorina respire, plus large. On rentre ? Oui. Les joues de Victorina se réchauffent. La carte reste froide sous la main. On le voit, maman. Tu le vois dans l'air ? Oui, l'éclat. Un &lt;emphasis&gt;éclat de poussière&lt;/emphasis&gt; reste pâle.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2030,18 +2080,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2050,12 +2100,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2064,17 +2114,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de poussière</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2083,11 +2137,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2096,29 +2150,50 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_pale; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|La poire claire brille sur le carton.
-enfant-f|J'ai regardé d'abord.
-copain|J'ai répété.
-maman|Puis la poire est arrivée.
-papa|Oui.
-narrateur|La clochette dort dans la chaussette.</t>
+          <t>enfant-f|Le rayon brillait, papa.
+papa|Tu le vois, comme dans l'air ?
+enfant-f|Oui, un peu pâle.
+narrateur|Victorina pose la carte contre le foulard.
+maman|On la garde près de nous ?
+enfant-f|Oui, maman.
+enfant-f|La classe sentait le bois.
+maman|Elle est derrière nous.
+narrateur|Un rayon n'est plus aussi net.
+narrateur|Victorina respire, plus large.
+papa|On rentre ?
+enfant-f|Oui.
+narrateur|Les joues de Victorina se réchauffent.
+narrateur|La carte reste froide sous la main.
+enfant-f|On le voit, maman.
+maman|Tu le vois dans l'air ?
+enfant-f|Oui, l'éclat.
+narrateur|Un éclat de poussière reste pâle.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>rayon</t>
         </is>
       </c>
     </row>
@@ -2139,7 +2214,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2217,6 +2292,13 @@
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>